<commit_message>
BOM Changes Completed Client BOM Bana dia ha TOP ,BOttom PCB ka
</commit_message>
<xml_diff>
--- a/Design-Files/SM_Bottom_Board/Project Outputs for SM_Bottom_Board/SM_Bottom_Board.xlsx
+++ b/Design-Files/SM_Bottom_Board/Project Outputs for SM_Bottom_Board/SM_Bottom_Board.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\ColeBenson-SmartMotors\Design-Files\SM_Bottom_Board\Project Outputs for SM_Bottom_Board\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\ColeBenson-SmartMotors\Design-Files\SM_Bottom_Board\Project Outputs for SM_Bottom_Board\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="2370" windowHeight="105"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22140" windowHeight="14430"/>
   </bookViews>
   <sheets>
     <sheet name="SM_Bottom_Board" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="164">
   <si>
     <t>Comment</t>
   </si>
@@ -146,7 +146,7 @@
     <t>TDK</t>
   </si>
   <si>
-    <t>10uF'</t>
+    <t>10uF</t>
   </si>
   <si>
     <t>CAP CER 10UF 25V X5R 0603</t>
@@ -194,10 +194,22 @@
     <t>ON Semiconductor</t>
   </si>
   <si>
-    <t>M55-6012042R</t>
-  </si>
-  <si>
-    <t>CONN RCPT 1.27MM DUAL SMD 20POS</t>
+    <t>MH254RS-11-02-1000</t>
+  </si>
+  <si>
+    <t>3A Surface Mount Header 1x2 SMD,P=2.54mm Pin Headers ROHS</t>
+  </si>
+  <si>
+    <t>J2</t>
+  </si>
+  <si>
+    <t>XFCN</t>
+  </si>
+  <si>
+    <t>M55-6012642R</t>
+  </si>
+  <si>
+    <t>CONN RCPT 26POS 0.05 GOLD SMD</t>
   </si>
   <si>
     <t>J3</t>
@@ -290,7 +302,7 @@
     <t>RES SMD 10K Ohm 1% 1/10W 0603</t>
   </si>
   <si>
-    <t>R2, R27, RF1, RF2, RF3</t>
+    <t>R2, R27, RF1, RF2, RF3, RF4, RF5</t>
   </si>
   <si>
     <t>RC0603FR-0710KL</t>
@@ -338,31 +350,25 @@
     <t>RC0603FR-07470RL</t>
   </si>
   <si>
-    <t>46R6</t>
-  </si>
-  <si>
-    <t>Res SMD 0603 46.4 Ohm 1% 1/10W</t>
+    <t>57R6</t>
+  </si>
+  <si>
+    <t>RES SMD 57.6 OHM 1% 1/10W 0603</t>
   </si>
   <si>
     <t>R7, R8</t>
   </si>
   <si>
-    <t>ERJ3EKF46R4V</t>
-  </si>
-  <si>
-    <t>Panasonic</t>
-  </si>
-  <si>
-    <t>ERJ-3EKF46R4V</t>
-  </si>
-  <si>
-    <t>RES SMD 1K OHM 1% 1/20W 0201</t>
-  </si>
-  <si>
-    <t>R9, R10</t>
-  </si>
-  <si>
-    <t>RC0201FR-071KL</t>
+    <t>RC0603FR-0757R6L</t>
+  </si>
+  <si>
+    <t>Solder Bridge</t>
+  </si>
+  <si>
+    <t>Solder Bridge ON</t>
+  </si>
+  <si>
+    <t>SB1</t>
   </si>
   <si>
     <t>B3U-1000P</t>
@@ -864,7 +870,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="10" width="16.5703125" customWidth="1"/>
@@ -1170,7 +1176,7 @@
       </c>
       <c r="J10" s="4"/>
     </row>
-    <row r="11" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>55</v>
       </c>
@@ -1193,12 +1199,10 @@
       <c r="H11" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="I11" s="3" t="s">
-        <v>55</v>
-      </c>
+      <c r="I11" s="4"/>
       <c r="J11" s="4"/>
     </row>
-    <row r="12" spans="1:10" ht="90" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>59</v>
       </c>
@@ -1209,7 +1213,7 @@
         <v>61</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>59</v>
@@ -1217,72 +1221,72 @@
       <c r="F12" s="4">
         <v>1</v>
       </c>
-      <c r="G12" s="3" t="s">
-        <v>15</v>
-      </c>
+      <c r="G12" s="4"/>
       <c r="H12" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I12" s="3" t="s">
         <v>59</v>
       </c>
       <c r="J12" s="4"/>
     </row>
-    <row r="13" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="90" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="C13" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="E13" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F13" s="4">
+        <v>1</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E13" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="F13" s="4">
-        <v>1</v>
-      </c>
-      <c r="G13" s="3" t="s">
+      <c r="I13" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="J13" s="4"/>
+    </row>
+    <row r="14" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="H13" s="3" t="s">
+      <c r="B14" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="I13" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="J13" s="4"/>
-    </row>
-    <row r="14" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
+      <c r="C14" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="D14" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="E14" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F14" s="4">
+        <v>1</v>
+      </c>
+      <c r="G14" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="F14" s="4">
-        <v>1</v>
-      </c>
-      <c r="G14" s="4"/>
       <c r="H14" s="3" t="s">
         <v>73</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="J14" s="4"/>
     </row>
@@ -1297,19 +1301,17 @@
         <v>76</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>74</v>
       </c>
       <c r="F15" s="4">
-        <v>2</v>
-      </c>
-      <c r="G15" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="G15" s="4"/>
+      <c r="H15" s="3" t="s">
         <v>77</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>78</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>74</v>
@@ -1318,65 +1320,65 @@
     </row>
     <row r="16" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="C16" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="D16" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="E16" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F16" s="4">
+        <v>2</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="H16" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="E16" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="F16" s="4">
-        <v>1</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>84</v>
-      </c>
       <c r="I16" s="3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="J16" s="4"/>
     </row>
     <row r="17" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="D17" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="E17" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="D17" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>88</v>
-      </c>
       <c r="F17" s="4">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>15</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J17" s="4"/>
     </row>
-    <row r="18" spans="1:10" ht="90" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>89</v>
       </c>
@@ -1387,52 +1389,52 @@
         <v>91</v>
       </c>
       <c r="D18" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E18" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="F18" s="4">
+        <v>7</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="J18" s="4"/>
+    </row>
+    <row r="19" spans="1:10" ht="90" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="F18" s="4">
-        <v>1</v>
-      </c>
-      <c r="G18" s="3" t="s">
+      <c r="B19" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="F19" s="4">
+        <v>1</v>
+      </c>
+      <c r="G19" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="H18" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="J18" s="4"/>
-    </row>
-    <row r="19" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="C19" s="3" t="s">
+      <c r="H19" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="I19" s="3" t="s">
         <v>97</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="F19" s="4">
-        <v>2</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="I19" s="3" t="s">
-        <v>98</v>
       </c>
       <c r="J19" s="4"/>
     </row>
@@ -1447,19 +1449,19 @@
         <v>101</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>102</v>
       </c>
       <c r="F20" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G20" s="3" t="s">
         <v>15</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="I20" s="3" t="s">
         <v>102</v>
@@ -1477,324 +1479,320 @@
         <v>105</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>106</v>
       </c>
       <c r="F21" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G21" s="3" t="s">
         <v>15</v>
       </c>
       <c r="H21" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="J21" s="4"/>
+    </row>
+    <row r="22" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="I21" s="3" t="s">
+      <c r="B22" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="J21" s="4"/>
-    </row>
-    <row r="22" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="B22" s="3" t="s">
+      <c r="C22" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="D22" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E22" s="3" t="s">
         <v>110</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>111</v>
       </c>
       <c r="F22" s="4">
         <v>2</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="I22" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="J22" s="4"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="J22" s="4"/>
-    </row>
-    <row r="23" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
+      <c r="B23" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="C23" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="C23" s="3" t="s">
-        <v>114</v>
-      </c>
       <c r="D23" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F23" s="4">
         <v>1</v>
       </c>
       <c r="G23" s="4"/>
-      <c r="H23" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="I23" s="3" t="s">
-        <v>112</v>
-      </c>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4"/>
       <c r="J23" s="4"/>
     </row>
     <row r="24" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C24" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="D24" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="F24" s="4">
+        <v>1</v>
+      </c>
+      <c r="G24" s="4"/>
+      <c r="H24" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="I24" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="J24" s="4"/>
+    </row>
+    <row r="25" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="B25" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="E24" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="F24" s="4">
-        <v>1</v>
-      </c>
-      <c r="G24" s="3" t="s">
+      <c r="C25" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="H24" s="3" t="s">
+      <c r="D25" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="I24" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="J24" s="4"/>
-    </row>
-    <row r="25" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
+      <c r="E25" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="F25" s="4">
+        <v>1</v>
+      </c>
+      <c r="G25" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="H25" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="I25" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="J25" s="4"/>
+    </row>
+    <row r="26" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="B26" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="E25" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="F25" s="4">
-        <v>1</v>
-      </c>
-      <c r="G25" s="4"/>
-      <c r="H25" s="3" t="s">
+      <c r="C26" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="I25" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="J25" s="4"/>
-    </row>
-    <row r="26" spans="1:10" ht="60" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
+      <c r="D26" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B26" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>130</v>
-      </c>
       <c r="E26" s="3" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="F26" s="4">
         <v>1</v>
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="I26" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="J26" s="4"/>
+    </row>
+    <row r="27" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C27" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="I26" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="J26" s="4"/>
-    </row>
-    <row r="27" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
+      <c r="D27" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="E27" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="F27" s="4">
+        <v>1</v>
+      </c>
+      <c r="G27" s="4"/>
+      <c r="H27" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="C27" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="F27" s="4">
-        <v>1</v>
-      </c>
-      <c r="G27" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="H27" s="3" t="s">
-        <v>137</v>
-      </c>
       <c r="I27" s="3" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="J27" s="4"/>
     </row>
     <row r="28" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="F28" s="4">
+        <v>1</v>
+      </c>
+      <c r="G28" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="H28" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="C28" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="F28" s="4">
-        <v>1</v>
-      </c>
-      <c r="G28" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="H28" s="3" t="s">
-        <v>126</v>
-      </c>
       <c r="I28" s="3" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="J28" s="4"/>
     </row>
     <row r="29" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C29" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="D29" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="C29" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>145</v>
-      </c>
       <c r="E29" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="F29" s="4">
         <v>1</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>147</v>
+        <v>128</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="J29" s="4"/>
     </row>
     <row r="30" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="F30" s="4">
+        <v>1</v>
+      </c>
+      <c r="G30" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="H30" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="C30" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="D30" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="F30" s="4">
-        <v>1</v>
-      </c>
-      <c r="G30" s="4"/>
-      <c r="H30" s="3" t="s">
-        <v>54</v>
-      </c>
       <c r="I30" s="3" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="J30" s="4"/>
     </row>
     <row r="31" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="C31" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="D31" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="C31" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="D31" s="3" t="s">
-        <v>155</v>
-      </c>
       <c r="E31" s="3" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="F31" s="4">
         <v>1</v>
       </c>
       <c r="G31" s="4"/>
       <c r="H31" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="I31" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="J31" s="4"/>
+    </row>
+    <row r="32" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="C32" s="3" t="s">
         <v>156</v>
-      </c>
-      <c r="I31" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="J31" s="4"/>
-    </row>
-    <row r="32" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>159</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>157</v>
@@ -1805,20 +1803,48 @@
       <c r="F32" s="4">
         <v>1</v>
       </c>
-      <c r="G32" s="3" t="s">
-        <v>160</v>
-      </c>
+      <c r="G32" s="4"/>
       <c r="H32" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="I32" s="3" t="s">
         <v>157</v>
       </c>
       <c r="J32" s="4"/>
+    </row>
+    <row r="33" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="F33" s="4">
+        <v>1</v>
+      </c>
+      <c r="G33" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="H33" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="I33" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="J33" s="4"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.30555555555555558" right="0.30555555555555558" top="0.30555555555555558" bottom="0.30555555555555558" header="0" footer="0"/>
-  <pageSetup scale="39" orientation="landscape" blackAndWhite="1" r:id="rId1"/>
+  <pageSetup scale="37" orientation="landscape" blackAndWhite="1" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>